<commit_message>
file/code(urban_district_upscaling\plain_scenario.xlsx): update column names for storage component
- column name "bus" is not needed anymore
- instead SESMG storage component requires "input" and "output"
</commit_message>
<xml_diff>
--- a/program_files/urban_district_upscaling/plain_scenario.xlsx
+++ b/program_files/urban_district_upscaling/plain_scenario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr updateLinks="never" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gregor/Desktop/Arbeit/Git/SESMG/program_files/urban_district_upscaling/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanBaumeister\Documents\GitHub\SESMG\program_files\urban_district_upscaling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AD6E57-C9C2-084E-AFAE-158F73A2D64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFCF889-9074-46E2-8051-0397316ADB6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18540" tabRatio="798" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="798" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="energysystem" sheetId="32" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="161">
   <si>
     <t>label</t>
   </si>
@@ -53,9 +53,6 @@
     <t>efficiency</t>
   </si>
   <si>
-    <t>bus</t>
-  </si>
-  <si>
     <t>initial capacity</t>
   </si>
   <si>
@@ -522,6 +519,9 @@
   </si>
   <si>
     <t>cleanliness</t>
+  </si>
+  <si>
+    <t>dc ac ratio</t>
   </si>
 </sst>
 </file>
@@ -1351,78 +1351,78 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25D30AE8-15DD-FE44-AC8F-03C9D89398A1}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="2" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.1640625" customWidth="1"/>
-    <col min="7" max="7" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" customWidth="1"/>
+    <col min="4" max="4" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.1796875" customWidth="1"/>
+    <col min="7" max="7" width="5.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="25" customFormat="1" ht="122">
+    <row r="1" spans="1:10" s="25" customFormat="1" ht="117">
       <c r="A1" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="C1" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="F1" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="D1" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="27" t="s">
-        <v>137</v>
-      </c>
       <c r="G1" s="27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H1" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="I1" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="I1" s="27" t="s">
+      <c r="J1" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="J1" s="27" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10">
+    </row>
+    <row r="2" spans="1:10" ht="13">
       <c r="A2" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1446,53 +1446,53 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3046EDF5-49B9-0E41-AB42-0AC2122A4A7B}">
   <dimension ref="A1:F50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="25" customFormat="1" ht="57">
+    <row r="1" spans="1:6" s="25" customFormat="1" ht="55">
       <c r="A1" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="C1" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="D1" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="E1" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="27" t="s">
-        <v>105</v>
-      </c>
       <c r="F1" s="27" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="13">
       <c r="A2" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1887,25 +1887,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F4561F9-8167-DF44-BCA9-B7DF3C27EBDA}">
   <dimension ref="A1:P50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="25" customFormat="1" ht="115">
+    <row r="1" spans="1:16" s="25" customFormat="1" ht="113">
       <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="26" t="s">
         <v>1</v>
@@ -1914,87 +1914,87 @@
         <v>2</v>
       </c>
       <c r="F1" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="28" t="s">
-        <v>32</v>
-      </c>
       <c r="H1" s="27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I1" s="26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J1" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="K1" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="L1" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="K1" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="L1" s="27" t="s">
+      <c r="N1" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="O1" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="P1" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="13">
+      <c r="A2" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="M1" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="N1" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="O1" s="26" t="s">
+      <c r="B2" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K2" s="74" t="s">
         <v>141</v>
       </c>
-      <c r="P1" s="27" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="K2" s="74" t="s">
-        <v>142</v>
-      </c>
       <c r="L2" s="74" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -2883,90 +2883,90 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED309585-3022-194C-9A97-AB7827FF4F22}">
   <dimension ref="A1:N50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.1796875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="8.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="25" customFormat="1" ht="65">
+    <row r="1" spans="1:14" s="25" customFormat="1" ht="62.5">
       <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F1" s="35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G1" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="I1" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="37" t="s">
-        <v>37</v>
-      </c>
       <c r="J1" s="38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K1" s="38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L1" s="71"/>
       <c r="M1" s="71"/>
       <c r="N1" s="71"/>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" ht="13">
       <c r="A2" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>39</v>
-      </c>
       <c r="K2" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -3609,274 +3609,281 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1390354-910C-204E-AADB-46606A5A746C}">
-  <dimension ref="A1:AL48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" outlineLevelCol="2"/>
+  <dimension ref="A1:AM48"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.1796875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="6" customWidth="1"/>
-    <col min="14" max="14" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="10" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="31" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="21" max="21" width="39.6640625" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="22" max="22" width="5.1640625" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="23" max="23" width="7.5" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="24" max="25" width="4.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="6.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="5.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="28" width="6.1640625" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="29" max="30" width="3.1640625" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="31" max="32" width="3.33203125" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="33" max="34" width="13.33203125" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="35" max="35" width="16.6640625" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="36" max="36" width="5.1640625" bestFit="1" customWidth="1" outlineLevel="2"/>
-    <col min="37" max="37" width="5.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="4.1640625" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="21" max="21" width="39.6328125" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="22" max="22" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="23" max="23" width="5.1796875" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="24" max="24" width="7.453125" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="26" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="6.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="28" width="5.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="29" max="29" width="6.1796875" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="30" max="31" width="3.1796875" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="32" max="33" width="3.36328125" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="34" max="35" width="13.36328125" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="36" max="36" width="16.6328125" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="37" max="37" width="5.1796875" bestFit="1" customWidth="1" outlineLevel="2"/>
+    <col min="38" max="38" width="5.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="39" max="39" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="25" customFormat="1" ht="119">
+    <row r="1" spans="1:39" s="25" customFormat="1" ht="115.5">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="36" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="J1" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="41" t="s">
+      <c r="K1" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="L1" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="M1" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="N1" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="P1" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="42" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="43" t="s">
-        <v>94</v>
-      </c>
-      <c r="M1" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="N1" s="43" t="s">
+      <c r="R1" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="S1" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="T1" s="46" t="s">
+        <v>144</v>
+      </c>
+      <c r="U1" s="46" t="s">
+        <v>145</v>
+      </c>
+      <c r="V1" s="46" t="s">
+        <v>160</v>
+      </c>
+      <c r="W1" s="46" t="s">
+        <v>146</v>
+      </c>
+      <c r="X1" s="46" t="s">
+        <v>147</v>
+      </c>
+      <c r="Y1" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="Z1" s="46" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA1" s="46" t="s">
+        <v>150</v>
+      </c>
+      <c r="AB1" s="46" t="s">
+        <v>151</v>
+      </c>
+      <c r="AC1" s="46" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD1" s="46" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE1" s="46" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF1" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="AG1" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH1" s="46" t="s">
+        <v>154</v>
+      </c>
+      <c r="AI1" s="46" t="s">
+        <v>155</v>
+      </c>
+      <c r="AJ1" s="46" t="s">
+        <v>156</v>
+      </c>
+      <c r="AK1" s="46" t="s">
+        <v>157</v>
+      </c>
+      <c r="AL1" s="46" t="s">
+        <v>158</v>
+      </c>
+      <c r="AM1" s="46" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:39" ht="13">
+      <c r="A2" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="48" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="L2" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="N2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="O1" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="P1" s="42" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q1" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="R1" s="37" t="s">
-        <v>153</v>
-      </c>
-      <c r="S1" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="T1" s="46" t="s">
-        <v>145</v>
-      </c>
-      <c r="U1" s="46" t="s">
-        <v>146</v>
-      </c>
-      <c r="V1" s="46" t="s">
-        <v>147</v>
-      </c>
-      <c r="W1" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="X1" s="46" t="s">
-        <v>149</v>
-      </c>
-      <c r="Y1" s="46" t="s">
-        <v>150</v>
-      </c>
-      <c r="Z1" s="46" t="s">
-        <v>151</v>
-      </c>
-      <c r="AA1" s="46" t="s">
-        <v>152</v>
-      </c>
-      <c r="AB1" s="46" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC1" s="46" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD1" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE1" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="AF1" s="46" t="s">
+      <c r="P2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="AG1" s="46" t="s">
-        <v>155</v>
-      </c>
-      <c r="AH1" s="46" t="s">
-        <v>156</v>
-      </c>
-      <c r="AI1" s="46" t="s">
-        <v>157</v>
-      </c>
-      <c r="AJ1" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="AK1" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="AL1" s="46" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="2" spans="1:38">
-      <c r="A2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="H2" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="48" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" s="49" t="s">
-        <v>131</v>
-      </c>
-      <c r="L2" s="50" t="s">
+      <c r="S2" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="T2" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="U2" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="V2" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="W2" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="X2" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y2" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z2" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA2" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB2" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC2" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="AD2" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="AE2" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="AF2" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="AG2" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="AH2" s="52" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI2" s="52" t="s">
+        <v>55</v>
+      </c>
+      <c r="AJ2" s="52" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK2" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="M2" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="N2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="P2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q2" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="R2" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="S2" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="T2" s="52" t="s">
-        <v>59</v>
-      </c>
-      <c r="U2" s="52" t="s">
-        <v>59</v>
-      </c>
-      <c r="V2" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="W2" s="52" t="s">
-        <v>60</v>
-      </c>
-      <c r="X2" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y2" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z2" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="AA2" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB2" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="AC2" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="AD2" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="AE2" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="AF2" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="AG2" s="52" t="s">
-        <v>56</v>
-      </c>
-      <c r="AH2" s="52" t="s">
-        <v>56</v>
-      </c>
-      <c r="AI2" s="52" t="s">
-        <v>57</v>
-      </c>
-      <c r="AJ2" s="52" t="s">
-        <v>49</v>
-      </c>
-      <c r="AK2" s="52" t="s">
-        <v>131</v>
-      </c>
       <c r="AL2" s="52" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="3" spans="1:38">
+        <v>130</v>
+      </c>
+      <c r="AM2" s="52" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:39">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -3915,8 +3922,9 @@
       <c r="AJ3" s="5"/>
       <c r="AK3" s="5"/>
       <c r="AL3" s="5"/>
-    </row>
-    <row r="4" spans="1:38">
+      <c r="AM3" s="5"/>
+    </row>
+    <row r="4" spans="1:39">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3955,8 +3963,9 @@
       <c r="AJ4" s="6"/>
       <c r="AK4" s="6"/>
       <c r="AL4" s="6"/>
-    </row>
-    <row r="5" spans="1:38">
+      <c r="AM4" s="6"/>
+    </row>
+    <row r="5" spans="1:39">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -3995,8 +4004,9 @@
       <c r="AJ5" s="5"/>
       <c r="AK5" s="5"/>
       <c r="AL5" s="5"/>
-    </row>
-    <row r="6" spans="1:38">
+      <c r="AM5" s="5"/>
+    </row>
+    <row r="6" spans="1:39">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4035,8 +4045,9 @@
       <c r="AJ6" s="6"/>
       <c r="AK6" s="6"/>
       <c r="AL6" s="6"/>
-    </row>
-    <row r="7" spans="1:38">
+      <c r="AM6" s="6"/>
+    </row>
+    <row r="7" spans="1:39">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -4075,8 +4086,9 @@
       <c r="AJ7" s="5"/>
       <c r="AK7" s="5"/>
       <c r="AL7" s="5"/>
-    </row>
-    <row r="8" spans="1:38">
+      <c r="AM7" s="5"/>
+    </row>
+    <row r="8" spans="1:39">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -4115,8 +4127,9 @@
       <c r="AJ8" s="6"/>
       <c r="AK8" s="6"/>
       <c r="AL8" s="6"/>
-    </row>
-    <row r="9" spans="1:38">
+      <c r="AM8" s="6"/>
+    </row>
+    <row r="9" spans="1:39">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -4155,8 +4168,9 @@
       <c r="AJ9" s="5"/>
       <c r="AK9" s="5"/>
       <c r="AL9" s="5"/>
-    </row>
-    <row r="10" spans="1:38">
+      <c r="AM9" s="5"/>
+    </row>
+    <row r="10" spans="1:39">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -4195,8 +4209,9 @@
       <c r="AJ10" s="6"/>
       <c r="AK10" s="6"/>
       <c r="AL10" s="6"/>
-    </row>
-    <row r="11" spans="1:38">
+      <c r="AM10" s="6"/>
+    </row>
+    <row r="11" spans="1:39">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -4235,8 +4250,9 @@
       <c r="AJ11" s="5"/>
       <c r="AK11" s="5"/>
       <c r="AL11" s="5"/>
-    </row>
-    <row r="12" spans="1:38">
+      <c r="AM11" s="5"/>
+    </row>
+    <row r="12" spans="1:39">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -4275,8 +4291,9 @@
       <c r="AJ12" s="6"/>
       <c r="AK12" s="6"/>
       <c r="AL12" s="6"/>
-    </row>
-    <row r="13" spans="1:38">
+      <c r="AM12" s="6"/>
+    </row>
+    <row r="13" spans="1:39">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -4315,8 +4332,9 @@
       <c r="AJ13" s="5"/>
       <c r="AK13" s="5"/>
       <c r="AL13" s="5"/>
-    </row>
-    <row r="14" spans="1:38">
+      <c r="AM13" s="5"/>
+    </row>
+    <row r="14" spans="1:39">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -4355,8 +4373,9 @@
       <c r="AJ14" s="6"/>
       <c r="AK14" s="6"/>
       <c r="AL14" s="6"/>
-    </row>
-    <row r="15" spans="1:38">
+      <c r="AM14" s="6"/>
+    </row>
+    <row r="15" spans="1:39">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -4395,8 +4414,9 @@
       <c r="AJ15" s="5"/>
       <c r="AK15" s="5"/>
       <c r="AL15" s="5"/>
-    </row>
-    <row r="16" spans="1:38">
+      <c r="AM15" s="5"/>
+    </row>
+    <row r="16" spans="1:39">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4435,8 +4455,9 @@
       <c r="AJ16" s="6"/>
       <c r="AK16" s="6"/>
       <c r="AL16" s="6"/>
-    </row>
-    <row r="17" spans="1:38">
+      <c r="AM16" s="6"/>
+    </row>
+    <row r="17" spans="1:39">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -4475,8 +4496,9 @@
       <c r="AJ17" s="5"/>
       <c r="AK17" s="5"/>
       <c r="AL17" s="5"/>
-    </row>
-    <row r="18" spans="1:38">
+      <c r="AM17" s="5"/>
+    </row>
+    <row r="18" spans="1:39">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -4515,8 +4537,9 @@
       <c r="AJ18" s="6"/>
       <c r="AK18" s="6"/>
       <c r="AL18" s="6"/>
-    </row>
-    <row r="19" spans="1:38">
+      <c r="AM18" s="6"/>
+    </row>
+    <row r="19" spans="1:39">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -4555,8 +4578,9 @@
       <c r="AJ19" s="5"/>
       <c r="AK19" s="5"/>
       <c r="AL19" s="5"/>
-    </row>
-    <row r="20" spans="1:38">
+      <c r="AM19" s="5"/>
+    </row>
+    <row r="20" spans="1:39">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -4595,8 +4619,9 @@
       <c r="AJ20" s="6"/>
       <c r="AK20" s="6"/>
       <c r="AL20" s="6"/>
-    </row>
-    <row r="21" spans="1:38">
+      <c r="AM20" s="6"/>
+    </row>
+    <row r="21" spans="1:39">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -4635,8 +4660,9 @@
       <c r="AJ21" s="5"/>
       <c r="AK21" s="5"/>
       <c r="AL21" s="5"/>
-    </row>
-    <row r="22" spans="1:38">
+      <c r="AM21" s="5"/>
+    </row>
+    <row r="22" spans="1:39">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -4675,8 +4701,9 @@
       <c r="AJ22" s="6"/>
       <c r="AK22" s="6"/>
       <c r="AL22" s="6"/>
-    </row>
-    <row r="23" spans="1:38">
+      <c r="AM22" s="6"/>
+    </row>
+    <row r="23" spans="1:39">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -4715,8 +4742,9 @@
       <c r="AJ23" s="5"/>
       <c r="AK23" s="5"/>
       <c r="AL23" s="5"/>
-    </row>
-    <row r="24" spans="1:38">
+      <c r="AM23" s="5"/>
+    </row>
+    <row r="24" spans="1:39">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -4755,8 +4783,9 @@
       <c r="AJ24" s="6"/>
       <c r="AK24" s="6"/>
       <c r="AL24" s="6"/>
-    </row>
-    <row r="25" spans="1:38">
+      <c r="AM24" s="6"/>
+    </row>
+    <row r="25" spans="1:39">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -4795,8 +4824,9 @@
       <c r="AJ25" s="5"/>
       <c r="AK25" s="5"/>
       <c r="AL25" s="5"/>
-    </row>
-    <row r="26" spans="1:38">
+      <c r="AM25" s="5"/>
+    </row>
+    <row r="26" spans="1:39">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -4835,8 +4865,9 @@
       <c r="AJ26" s="6"/>
       <c r="AK26" s="6"/>
       <c r="AL26" s="6"/>
-    </row>
-    <row r="27" spans="1:38">
+      <c r="AM26" s="6"/>
+    </row>
+    <row r="27" spans="1:39">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -4875,8 +4906,9 @@
       <c r="AJ27" s="5"/>
       <c r="AK27" s="5"/>
       <c r="AL27" s="5"/>
-    </row>
-    <row r="28" spans="1:38">
+      <c r="AM27" s="5"/>
+    </row>
+    <row r="28" spans="1:39">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -4915,8 +4947,9 @@
       <c r="AJ28" s="6"/>
       <c r="AK28" s="6"/>
       <c r="AL28" s="6"/>
-    </row>
-    <row r="29" spans="1:38">
+      <c r="AM28" s="6"/>
+    </row>
+    <row r="29" spans="1:39">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -4955,8 +4988,9 @@
       <c r="AJ29" s="5"/>
       <c r="AK29" s="5"/>
       <c r="AL29" s="5"/>
-    </row>
-    <row r="30" spans="1:38">
+      <c r="AM29" s="5"/>
+    </row>
+    <row r="30" spans="1:39">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -4995,8 +5029,9 @@
       <c r="AJ30" s="6"/>
       <c r="AK30" s="6"/>
       <c r="AL30" s="6"/>
-    </row>
-    <row r="31" spans="1:38">
+      <c r="AM30" s="6"/>
+    </row>
+    <row r="31" spans="1:39">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -5035,8 +5070,9 @@
       <c r="AJ31" s="5"/>
       <c r="AK31" s="5"/>
       <c r="AL31" s="5"/>
-    </row>
-    <row r="32" spans="1:38">
+      <c r="AM31" s="5"/>
+    </row>
+    <row r="32" spans="1:39">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -5075,8 +5111,9 @@
       <c r="AJ32" s="6"/>
       <c r="AK32" s="6"/>
       <c r="AL32" s="6"/>
-    </row>
-    <row r="33" spans="1:38">
+      <c r="AM32" s="6"/>
+    </row>
+    <row r="33" spans="1:39">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -5115,8 +5152,9 @@
       <c r="AJ33" s="5"/>
       <c r="AK33" s="5"/>
       <c r="AL33" s="5"/>
-    </row>
-    <row r="34" spans="1:38">
+      <c r="AM33" s="5"/>
+    </row>
+    <row r="34" spans="1:39">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -5155,8 +5193,9 @@
       <c r="AJ34" s="6"/>
       <c r="AK34" s="6"/>
       <c r="AL34" s="6"/>
-    </row>
-    <row r="35" spans="1:38">
+      <c r="AM34" s="6"/>
+    </row>
+    <row r="35" spans="1:39">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -5195,8 +5234,9 @@
       <c r="AJ35" s="5"/>
       <c r="AK35" s="5"/>
       <c r="AL35" s="5"/>
-    </row>
-    <row r="36" spans="1:38">
+      <c r="AM35" s="5"/>
+    </row>
+    <row r="36" spans="1:39">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -5235,8 +5275,9 @@
       <c r="AJ36" s="6"/>
       <c r="AK36" s="6"/>
       <c r="AL36" s="6"/>
-    </row>
-    <row r="37" spans="1:38">
+      <c r="AM36" s="6"/>
+    </row>
+    <row r="37" spans="1:39">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -5275,8 +5316,9 @@
       <c r="AJ37" s="5"/>
       <c r="AK37" s="5"/>
       <c r="AL37" s="5"/>
-    </row>
-    <row r="38" spans="1:38">
+      <c r="AM37" s="5"/>
+    </row>
+    <row r="38" spans="1:39">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -5315,8 +5357,9 @@
       <c r="AJ38" s="6"/>
       <c r="AK38" s="6"/>
       <c r="AL38" s="6"/>
-    </row>
-    <row r="39" spans="1:38">
+      <c r="AM38" s="6"/>
+    </row>
+    <row r="39" spans="1:39">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -5355,8 +5398,9 @@
       <c r="AJ39" s="5"/>
       <c r="AK39" s="5"/>
       <c r="AL39" s="5"/>
-    </row>
-    <row r="40" spans="1:38">
+      <c r="AM39" s="5"/>
+    </row>
+    <row r="40" spans="1:39">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -5395,8 +5439,9 @@
       <c r="AJ40" s="6"/>
       <c r="AK40" s="6"/>
       <c r="AL40" s="6"/>
-    </row>
-    <row r="41" spans="1:38">
+      <c r="AM40" s="6"/>
+    </row>
+    <row r="41" spans="1:39">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -5435,8 +5480,9 @@
       <c r="AJ41" s="5"/>
       <c r="AK41" s="5"/>
       <c r="AL41" s="5"/>
-    </row>
-    <row r="42" spans="1:38">
+      <c r="AM41" s="5"/>
+    </row>
+    <row r="42" spans="1:39">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -5475,8 +5521,9 @@
       <c r="AJ42" s="6"/>
       <c r="AK42" s="6"/>
       <c r="AL42" s="6"/>
-    </row>
-    <row r="43" spans="1:38">
+      <c r="AM42" s="6"/>
+    </row>
+    <row r="43" spans="1:39">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -5515,8 +5562,9 @@
       <c r="AJ43" s="5"/>
       <c r="AK43" s="5"/>
       <c r="AL43" s="5"/>
-    </row>
-    <row r="44" spans="1:38">
+      <c r="AM43" s="5"/>
+    </row>
+    <row r="44" spans="1:39">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -5555,8 +5603,9 @@
       <c r="AJ44" s="6"/>
       <c r="AK44" s="6"/>
       <c r="AL44" s="6"/>
-    </row>
-    <row r="45" spans="1:38">
+      <c r="AM44" s="6"/>
+    </row>
+    <row r="45" spans="1:39">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -5595,8 +5644,9 @@
       <c r="AJ45" s="5"/>
       <c r="AK45" s="5"/>
       <c r="AL45" s="5"/>
-    </row>
-    <row r="46" spans="1:38">
+      <c r="AM45" s="5"/>
+    </row>
+    <row r="46" spans="1:39">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -5635,8 +5685,9 @@
       <c r="AJ46" s="6"/>
       <c r="AK46" s="6"/>
       <c r="AL46" s="6"/>
-    </row>
-    <row r="47" spans="1:38">
+      <c r="AM46" s="6"/>
+    </row>
+    <row r="47" spans="1:39">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -5675,8 +5726,9 @@
       <c r="AJ47" s="5"/>
       <c r="AK47" s="5"/>
       <c r="AL47" s="5"/>
-    </row>
-    <row r="48" spans="1:38">
+      <c r="AM47" s="5"/>
+    </row>
+    <row r="48" spans="1:39">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -5715,6 +5767,7 @@
       <c r="AJ48" s="6"/>
       <c r="AK48" s="6"/>
       <c r="AL48" s="6"/>
+      <c r="AM48" s="6"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C3:D48">
@@ -5733,40 +5786,40 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{202E8141-8F15-FF4E-A8C0-0B7CE02C7F8D}">
   <dimension ref="A1:AV46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" outlineLevelCol="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="12.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="2" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.1796875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="6" customWidth="1"/>
-    <col min="17" max="19" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="23" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.5" customWidth="1"/>
+    <col min="17" max="19" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="23" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.453125" customWidth="1"/>
     <col min="25" max="25" width="7" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="28" width="4.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="29" max="29" width="5.5" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="30" max="30" width="4.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="31" max="31" width="9.33203125" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="32" max="32" width="4.33203125" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="4.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="34" max="34" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="6.33203125" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="37" width="4.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="5.1640625" bestFit="1" customWidth="1" outlineLevel="1"/>
-    <col min="39" max="41" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="47" max="48" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="29" max="29" width="5.453125" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="30" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="31" max="31" width="9.36328125" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="32" max="32" width="4.36328125" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="34" max="34" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="6.36328125" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="36" max="37" width="4.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="38" width="5.1796875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="39" max="41" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="42" max="43" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="44" max="45" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="47" max="48" width="4.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:48" s="25" customFormat="1" ht="93" customHeight="1">
@@ -5774,291 +5827,291 @@
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F1" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="H1" s="36" t="s">
         <v>20</v>
-      </c>
-      <c r="H1" s="36" t="s">
-        <v>21</v>
       </c>
       <c r="I1" s="36" t="s">
         <v>3</v>
       </c>
       <c r="J1" s="59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K1" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="L1" s="40" t="s">
+      <c r="M1" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="M1" s="45" t="s">
+      <c r="N1" s="43" t="s">
+        <v>92</v>
+      </c>
+      <c r="O1" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="P1" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q1" s="43" t="s">
+        <v>11</v>
+      </c>
+      <c r="R1" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="S1" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="T1" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="U1" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="V1" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="W1" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="X1" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="43" t="s">
-        <v>93</v>
-      </c>
-      <c r="O1" s="43" t="s">
-        <v>94</v>
-      </c>
-      <c r="P1" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q1" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="R1" s="43" t="s">
-        <v>13</v>
-      </c>
-      <c r="S1" s="43" t="s">
-        <v>61</v>
-      </c>
-      <c r="T1" s="45" t="s">
-        <v>43</v>
-      </c>
-      <c r="U1" s="43" t="s">
-        <v>62</v>
-      </c>
-      <c r="V1" s="43" t="s">
-        <v>63</v>
-      </c>
-      <c r="W1" s="43" t="s">
+      <c r="Y1" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="X1" s="45" t="s">
+      <c r="Z1" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA1" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB1" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="AC1" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="AD1" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="AE1" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="AF1" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="AG1" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="AH1" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="AI1" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="AJ1" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="AK1" s="46" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL1" s="46" t="s">
+        <v>80</v>
+      </c>
+      <c r="AM1" s="46" t="s">
+        <v>81</v>
+      </c>
+      <c r="AN1" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="AO1" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="AP1" s="60" t="s">
+        <v>112</v>
+      </c>
+      <c r="AQ1" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="AR1" s="60" t="s">
+        <v>114</v>
+      </c>
+      <c r="AS1" s="60" t="s">
+        <v>115</v>
+      </c>
+      <c r="AT1" s="60" t="s">
+        <v>116</v>
+      </c>
+      <c r="AU1" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="AV1" s="60" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:48" ht="13">
+      <c r="A2" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="61" t="s">
+        <v>130</v>
+      </c>
+      <c r="K2" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="N2" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="O2" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="Y1" s="37" t="s">
-        <v>65</v>
-      </c>
-      <c r="Z1" s="37" t="s">
+      <c r="P2" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="W2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="X2" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y2" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="Z2" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="AA1" s="37" t="s">
-        <v>68</v>
-      </c>
-      <c r="AB1" s="37" t="s">
-        <v>69</v>
-      </c>
-      <c r="AC1" s="37" t="s">
+      <c r="AA2" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB2" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="AC2" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="AD1" s="37" t="s">
-        <v>100</v>
-      </c>
-      <c r="AE1" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="AF1" s="37" t="s">
-        <v>75</v>
-      </c>
-      <c r="AG1" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="AH1" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="AI1" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="AJ1" s="46" t="s">
-        <v>79</v>
-      </c>
-      <c r="AK1" s="46" t="s">
-        <v>80</v>
-      </c>
-      <c r="AL1" s="46" t="s">
-        <v>81</v>
-      </c>
-      <c r="AM1" s="46" t="s">
-        <v>82</v>
-      </c>
-      <c r="AN1" s="60" t="s">
-        <v>111</v>
-      </c>
-      <c r="AO1" s="60" t="s">
-        <v>112</v>
-      </c>
-      <c r="AP1" s="60" t="s">
-        <v>113</v>
-      </c>
-      <c r="AQ1" s="60" t="s">
-        <v>114</v>
-      </c>
-      <c r="AR1" s="60" t="s">
-        <v>115</v>
-      </c>
-      <c r="AS1" s="60" t="s">
-        <v>116</v>
-      </c>
-      <c r="AT1" s="60" t="s">
-        <v>117</v>
-      </c>
-      <c r="AU1" s="60" t="s">
-        <v>118</v>
-      </c>
-      <c r="AV1" s="60" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:48">
-      <c r="A2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="J2" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="K2" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="L2" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" s="51" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="O2" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="P2" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="R2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="S2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="T2" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="U2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="V2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="W2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="X2" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y2" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="Z2" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA2" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB2" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="AC2" s="15" t="s">
+      <c r="AD2" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="AD2" s="15" t="s">
+      <c r="AE2" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="AE2" s="15" t="s">
-        <v>73</v>
-      </c>
       <c r="AF2" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AG2" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AH2" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AI2" s="53" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AJ2" s="53" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AK2" s="53" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL2" s="53" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM2" s="53" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AN2" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AO2" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AP2" s="63" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AQ2" s="63" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AR2" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AS2" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AT2" s="63" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AU2" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AV2" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:48">
@@ -8278,212 +8331,218 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33FA34E7-A3CF-AE49-853F-E47D76E2EEDF}">
-  <dimension ref="A1:AC50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <dimension ref="A1:AD50"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.5" customWidth="1"/>
-    <col min="19" max="20" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" customWidth="1"/>
-    <col min="28" max="28" width="8.83203125" customWidth="1"/>
-    <col min="29" max="29" width="27.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.453125" customWidth="1"/>
+    <col min="20" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.81640625" customWidth="1"/>
+    <col min="29" max="29" width="8.81640625" customWidth="1"/>
+    <col min="30" max="30" width="27.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="122">
+    <row r="1" spans="1:30" ht="118.5">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="I1" s="36" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="36" t="s">
+        <v>5</v>
+      </c>
+      <c r="M1" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="O1" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="P1" s="66" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q1" s="67" t="s">
+        <v>92</v>
+      </c>
+      <c r="R1" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="S1" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="T1" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="U1" s="36" t="s">
+        <v>12</v>
+      </c>
+      <c r="V1" s="66" t="s">
+        <v>42</v>
+      </c>
+      <c r="W1" s="67" t="s">
+        <v>61</v>
+      </c>
+      <c r="X1" s="36" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y1" s="66" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z1" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA1" s="46" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB1" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC1" s="46" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD1" s="46" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" ht="13">
+      <c r="A2" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="M2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="N2" s="47" t="s">
+        <v>91</v>
+      </c>
+      <c r="O2" s="47" t="s">
+        <v>91</v>
+      </c>
+      <c r="P2" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q2" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="R2" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="S2" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="T2" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="36" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="H1" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="36" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="36" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="N1" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="O1" s="66" t="s">
-        <v>46</v>
-      </c>
-      <c r="P1" s="67" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q1" s="36" t="s">
-        <v>94</v>
-      </c>
-      <c r="R1" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="S1" s="36" t="s">
-        <v>12</v>
-      </c>
-      <c r="T1" s="36" t="s">
-        <v>13</v>
-      </c>
-      <c r="U1" s="66" t="s">
-        <v>43</v>
-      </c>
-      <c r="V1" s="67" t="s">
-        <v>62</v>
-      </c>
-      <c r="W1" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="X1" s="66" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y1" s="37" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z1" s="46" t="s">
-        <v>95</v>
-      </c>
-      <c r="AA1" s="46" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB1" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC1" s="46" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29">
-      <c r="A2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="K2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="M2" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="N2" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="O2" s="51" t="s">
-        <v>92</v>
-      </c>
-      <c r="P2" s="49" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q2" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="R2" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="S2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="T2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="U2" s="68" t="s">
-        <v>83</v>
-      </c>
-      <c r="V2" s="49" t="s">
-        <v>29</v>
-      </c>
-      <c r="W2" s="50" t="s">
-        <v>29</v>
-      </c>
-      <c r="X2" s="68" t="s">
-        <v>83</v>
-      </c>
-      <c r="Y2" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="Z2" s="53" t="s">
-        <v>89</v>
+      <c r="U2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" s="68" t="s">
+        <v>82</v>
+      </c>
+      <c r="W2" s="49" t="s">
+        <v>28</v>
+      </c>
+      <c r="X2" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y2" s="68" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z2" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="AA2" s="53" t="s">
         <v>88</v>
       </c>
       <c r="AB2" s="53" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AC2" s="53" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29">
+        <v>87</v>
+      </c>
+      <c r="AD2" s="53" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -8496,25 +8555,26 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="9"/>
+      <c r="M3" s="1"/>
       <c r="N3" s="9"/>
-      <c r="O3" s="55"/>
-      <c r="P3" s="54"/>
-      <c r="Q3" s="1"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="55"/>
+      <c r="Q3" s="54"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="54"/>
-      <c r="W3" s="1"/>
-      <c r="X3" s="20"/>
-      <c r="Y3" s="7"/>
-      <c r="Z3" s="69"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="20"/>
+      <c r="W3" s="54"/>
+      <c r="X3" s="1"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="7"/>
       <c r="AA3" s="69"/>
       <c r="AB3" s="69"/>
       <c r="AC3" s="69"/>
-    </row>
-    <row r="4" spans="1:29">
+      <c r="AD3" s="69"/>
+    </row>
+    <row r="4" spans="1:30">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -8527,25 +8587,26 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
-      <c r="M4" s="10"/>
+      <c r="M4" s="2"/>
       <c r="N4" s="10"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="2"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="57"/>
+      <c r="Q4" s="56"/>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
-      <c r="U4" s="18"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="18"/>
-      <c r="Y4" s="8"/>
-      <c r="Z4" s="70"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="18"/>
+      <c r="W4" s="56"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="18"/>
+      <c r="Z4" s="8"/>
       <c r="AA4" s="70"/>
       <c r="AB4" s="70"/>
       <c r="AC4" s="70"/>
-    </row>
-    <row r="5" spans="1:29">
+      <c r="AD4" s="70"/>
+    </row>
+    <row r="5" spans="1:30">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -8558,25 +8619,26 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="9"/>
+      <c r="M5" s="1"/>
       <c r="N5" s="9"/>
-      <c r="O5" s="55"/>
-      <c r="P5" s="54"/>
-      <c r="Q5" s="1"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="54"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="54"/>
-      <c r="W5" s="1"/>
-      <c r="X5" s="20"/>
-      <c r="Y5" s="7"/>
-      <c r="Z5" s="69"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="54"/>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="7"/>
       <c r="AA5" s="69"/>
       <c r="AB5" s="69"/>
       <c r="AC5" s="69"/>
-    </row>
-    <row r="6" spans="1:29">
+      <c r="AD5" s="69"/>
+    </row>
+    <row r="6" spans="1:30">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -8589,25 +8651,26 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="M6" s="10"/>
+      <c r="M6" s="2"/>
       <c r="N6" s="10"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="2"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="57"/>
+      <c r="Q6" s="56"/>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="56"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="18"/>
-      <c r="Y6" s="8"/>
-      <c r="Z6" s="70"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="56"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="8"/>
       <c r="AA6" s="70"/>
       <c r="AB6" s="70"/>
       <c r="AC6" s="70"/>
-    </row>
-    <row r="7" spans="1:29">
+      <c r="AD6" s="70"/>
+    </row>
+    <row r="7" spans="1:30">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -8620,25 +8683,26 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
-      <c r="M7" s="9"/>
+      <c r="M7" s="1"/>
       <c r="N7" s="9"/>
-      <c r="O7" s="55"/>
-      <c r="P7" s="54"/>
-      <c r="Q7" s="1"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="55"/>
+      <c r="Q7" s="54"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="54"/>
-      <c r="W7" s="1"/>
-      <c r="X7" s="20"/>
-      <c r="Y7" s="7"/>
-      <c r="Z7" s="69"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="54"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="20"/>
+      <c r="Z7" s="7"/>
       <c r="AA7" s="69"/>
       <c r="AB7" s="69"/>
       <c r="AC7" s="69"/>
-    </row>
-    <row r="8" spans="1:29">
+      <c r="AD7" s="69"/>
+    </row>
+    <row r="8" spans="1:30">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -8651,25 +8715,26 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-      <c r="M8" s="10"/>
+      <c r="M8" s="2"/>
       <c r="N8" s="10"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="56"/>
-      <c r="Q8" s="2"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="57"/>
+      <c r="Q8" s="56"/>
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
-      <c r="U8" s="18"/>
-      <c r="V8" s="56"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="18"/>
-      <c r="Y8" s="8"/>
-      <c r="Z8" s="70"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="18"/>
+      <c r="W8" s="56"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="18"/>
+      <c r="Z8" s="8"/>
       <c r="AA8" s="70"/>
       <c r="AB8" s="70"/>
       <c r="AC8" s="70"/>
-    </row>
-    <row r="9" spans="1:29">
+      <c r="AD8" s="70"/>
+    </row>
+    <row r="9" spans="1:30">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -8682,25 +8747,26 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="9"/>
+      <c r="M9" s="1"/>
       <c r="N9" s="9"/>
-      <c r="O9" s="55"/>
-      <c r="P9" s="54"/>
-      <c r="Q9" s="1"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="55"/>
+      <c r="Q9" s="54"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="54"/>
-      <c r="W9" s="1"/>
-      <c r="X9" s="20"/>
-      <c r="Y9" s="7"/>
-      <c r="Z9" s="69"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="20"/>
+      <c r="W9" s="54"/>
+      <c r="X9" s="1"/>
+      <c r="Y9" s="20"/>
+      <c r="Z9" s="7"/>
       <c r="AA9" s="69"/>
       <c r="AB9" s="69"/>
       <c r="AC9" s="69"/>
-    </row>
-    <row r="10" spans="1:29">
+      <c r="AD9" s="69"/>
+    </row>
+    <row r="10" spans="1:30">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -8713,25 +8779,26 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
-      <c r="M10" s="10"/>
+      <c r="M10" s="2"/>
       <c r="N10" s="10"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="56"/>
-      <c r="Q10" s="2"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="57"/>
+      <c r="Q10" s="56"/>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
-      <c r="U10" s="18"/>
-      <c r="V10" s="56"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="18"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="70"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="18"/>
+      <c r="W10" s="56"/>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="18"/>
+      <c r="Z10" s="8"/>
       <c r="AA10" s="70"/>
       <c r="AB10" s="70"/>
       <c r="AC10" s="70"/>
-    </row>
-    <row r="11" spans="1:29">
+      <c r="AD10" s="70"/>
+    </row>
+    <row r="11" spans="1:30">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -8744,25 +8811,26 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
-      <c r="M11" s="9"/>
+      <c r="M11" s="1"/>
       <c r="N11" s="9"/>
-      <c r="O11" s="55"/>
-      <c r="P11" s="54"/>
-      <c r="Q11" s="1"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="55"/>
+      <c r="Q11" s="54"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="54"/>
-      <c r="W11" s="1"/>
-      <c r="X11" s="20"/>
-      <c r="Y11" s="7"/>
-      <c r="Z11" s="69"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="20"/>
+      <c r="W11" s="54"/>
+      <c r="X11" s="1"/>
+      <c r="Y11" s="20"/>
+      <c r="Z11" s="7"/>
       <c r="AA11" s="69"/>
       <c r="AB11" s="69"/>
       <c r="AC11" s="69"/>
-    </row>
-    <row r="12" spans="1:29">
+      <c r="AD11" s="69"/>
+    </row>
+    <row r="12" spans="1:30">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -8775,25 +8843,26 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="10"/>
+      <c r="M12" s="2"/>
       <c r="N12" s="10"/>
-      <c r="O12" s="57"/>
-      <c r="P12" s="56"/>
-      <c r="Q12" s="2"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="57"/>
+      <c r="Q12" s="56"/>
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
-      <c r="U12" s="18"/>
-      <c r="V12" s="56"/>
-      <c r="W12" s="2"/>
-      <c r="X12" s="18"/>
-      <c r="Y12" s="8"/>
-      <c r="Z12" s="70"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="18"/>
+      <c r="W12" s="56"/>
+      <c r="X12" s="2"/>
+      <c r="Y12" s="18"/>
+      <c r="Z12" s="8"/>
       <c r="AA12" s="70"/>
       <c r="AB12" s="70"/>
       <c r="AC12" s="70"/>
-    </row>
-    <row r="13" spans="1:29">
+      <c r="AD12" s="70"/>
+    </row>
+    <row r="13" spans="1:30">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -8806,25 +8875,26 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
-      <c r="M13" s="9"/>
+      <c r="M13" s="1"/>
       <c r="N13" s="9"/>
-      <c r="O13" s="55"/>
-      <c r="P13" s="54"/>
-      <c r="Q13" s="1"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="55"/>
+      <c r="Q13" s="54"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
-      <c r="U13" s="20"/>
-      <c r="V13" s="54"/>
-      <c r="W13" s="1"/>
-      <c r="X13" s="20"/>
-      <c r="Y13" s="7"/>
-      <c r="Z13" s="69"/>
+      <c r="U13" s="1"/>
+      <c r="V13" s="20"/>
+      <c r="W13" s="54"/>
+      <c r="X13" s="1"/>
+      <c r="Y13" s="20"/>
+      <c r="Z13" s="7"/>
       <c r="AA13" s="69"/>
       <c r="AB13" s="69"/>
       <c r="AC13" s="69"/>
-    </row>
-    <row r="14" spans="1:29">
+      <c r="AD13" s="69"/>
+    </row>
+    <row r="14" spans="1:30">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -8837,25 +8907,26 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
-      <c r="M14" s="10"/>
+      <c r="M14" s="2"/>
       <c r="N14" s="10"/>
-      <c r="O14" s="57"/>
-      <c r="P14" s="56"/>
-      <c r="Q14" s="2"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="57"/>
+      <c r="Q14" s="56"/>
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
-      <c r="U14" s="18"/>
-      <c r="V14" s="56"/>
-      <c r="W14" s="2"/>
-      <c r="X14" s="18"/>
-      <c r="Y14" s="8"/>
-      <c r="Z14" s="70"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="18"/>
+      <c r="W14" s="56"/>
+      <c r="X14" s="2"/>
+      <c r="Y14" s="18"/>
+      <c r="Z14" s="8"/>
       <c r="AA14" s="70"/>
       <c r="AB14" s="70"/>
       <c r="AC14" s="70"/>
-    </row>
-    <row r="15" spans="1:29">
+      <c r="AD14" s="70"/>
+    </row>
+    <row r="15" spans="1:30">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -8868,25 +8939,26 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
-      <c r="M15" s="9"/>
+      <c r="M15" s="1"/>
       <c r="N15" s="9"/>
-      <c r="O15" s="55"/>
-      <c r="P15" s="54"/>
-      <c r="Q15" s="1"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="55"/>
+      <c r="Q15" s="54"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
-      <c r="U15" s="20"/>
-      <c r="V15" s="54"/>
-      <c r="W15" s="1"/>
-      <c r="X15" s="20"/>
-      <c r="Y15" s="7"/>
-      <c r="Z15" s="69"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="20"/>
+      <c r="W15" s="54"/>
+      <c r="X15" s="1"/>
+      <c r="Y15" s="20"/>
+      <c r="Z15" s="7"/>
       <c r="AA15" s="69"/>
       <c r="AB15" s="69"/>
       <c r="AC15" s="69"/>
-    </row>
-    <row r="16" spans="1:29">
+      <c r="AD15" s="69"/>
+    </row>
+    <row r="16" spans="1:30">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -8899,25 +8971,26 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
-      <c r="M16" s="10"/>
+      <c r="M16" s="2"/>
       <c r="N16" s="10"/>
-      <c r="O16" s="57"/>
-      <c r="P16" s="56"/>
-      <c r="Q16" s="2"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="57"/>
+      <c r="Q16" s="56"/>
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
-      <c r="U16" s="18"/>
-      <c r="V16" s="56"/>
-      <c r="W16" s="2"/>
-      <c r="X16" s="18"/>
-      <c r="Y16" s="8"/>
-      <c r="Z16" s="70"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="18"/>
+      <c r="W16" s="56"/>
+      <c r="X16" s="2"/>
+      <c r="Y16" s="18"/>
+      <c r="Z16" s="8"/>
       <c r="AA16" s="70"/>
       <c r="AB16" s="70"/>
       <c r="AC16" s="70"/>
-    </row>
-    <row r="17" spans="1:29">
+      <c r="AD16" s="70"/>
+    </row>
+    <row r="17" spans="1:30">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -8930,25 +9003,26 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
-      <c r="M17" s="9"/>
+      <c r="M17" s="1"/>
       <c r="N17" s="9"/>
-      <c r="O17" s="55"/>
-      <c r="P17" s="54"/>
-      <c r="Q17" s="1"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="55"/>
+      <c r="Q17" s="54"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
-      <c r="U17" s="20"/>
-      <c r="V17" s="54"/>
-      <c r="W17" s="1"/>
-      <c r="X17" s="20"/>
-      <c r="Y17" s="7"/>
-      <c r="Z17" s="69"/>
+      <c r="U17" s="1"/>
+      <c r="V17" s="20"/>
+      <c r="W17" s="54"/>
+      <c r="X17" s="1"/>
+      <c r="Y17" s="20"/>
+      <c r="Z17" s="7"/>
       <c r="AA17" s="69"/>
       <c r="AB17" s="69"/>
       <c r="AC17" s="69"/>
-    </row>
-    <row r="18" spans="1:29">
+      <c r="AD17" s="69"/>
+    </row>
+    <row r="18" spans="1:30">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -8961,25 +9035,26 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
-      <c r="M18" s="10"/>
+      <c r="M18" s="2"/>
       <c r="N18" s="10"/>
-      <c r="O18" s="57"/>
-      <c r="P18" s="56"/>
-      <c r="Q18" s="2"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="57"/>
+      <c r="Q18" s="56"/>
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
-      <c r="U18" s="18"/>
-      <c r="V18" s="56"/>
-      <c r="W18" s="2"/>
-      <c r="X18" s="18"/>
-      <c r="Y18" s="8"/>
-      <c r="Z18" s="70"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="18"/>
+      <c r="W18" s="56"/>
+      <c r="X18" s="2"/>
+      <c r="Y18" s="18"/>
+      <c r="Z18" s="8"/>
       <c r="AA18" s="70"/>
       <c r="AB18" s="70"/>
       <c r="AC18" s="70"/>
-    </row>
-    <row r="19" spans="1:29">
+      <c r="AD18" s="70"/>
+    </row>
+    <row r="19" spans="1:30">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -8992,25 +9067,26 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
-      <c r="M19" s="9"/>
+      <c r="M19" s="1"/>
       <c r="N19" s="9"/>
-      <c r="O19" s="55"/>
-      <c r="P19" s="54"/>
-      <c r="Q19" s="1"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="55"/>
+      <c r="Q19" s="54"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
-      <c r="U19" s="20"/>
-      <c r="V19" s="54"/>
-      <c r="W19" s="1"/>
-      <c r="X19" s="20"/>
-      <c r="Y19" s="7"/>
-      <c r="Z19" s="69"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="20"/>
+      <c r="W19" s="54"/>
+      <c r="X19" s="1"/>
+      <c r="Y19" s="20"/>
+      <c r="Z19" s="7"/>
       <c r="AA19" s="69"/>
       <c r="AB19" s="69"/>
       <c r="AC19" s="69"/>
-    </row>
-    <row r="20" spans="1:29">
+      <c r="AD19" s="69"/>
+    </row>
+    <row r="20" spans="1:30">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -9023,25 +9099,26 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
-      <c r="M20" s="10"/>
+      <c r="M20" s="2"/>
       <c r="N20" s="10"/>
-      <c r="O20" s="57"/>
-      <c r="P20" s="56"/>
-      <c r="Q20" s="2"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="57"/>
+      <c r="Q20" s="56"/>
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
       <c r="T20" s="2"/>
-      <c r="U20" s="18"/>
-      <c r="V20" s="56"/>
-      <c r="W20" s="2"/>
-      <c r="X20" s="18"/>
-      <c r="Y20" s="8"/>
-      <c r="Z20" s="70"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="18"/>
+      <c r="W20" s="56"/>
+      <c r="X20" s="2"/>
+      <c r="Y20" s="18"/>
+      <c r="Z20" s="8"/>
       <c r="AA20" s="70"/>
       <c r="AB20" s="70"/>
       <c r="AC20" s="70"/>
-    </row>
-    <row r="21" spans="1:29">
+      <c r="AD20" s="70"/>
+    </row>
+    <row r="21" spans="1:30">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -9054,25 +9131,26 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
-      <c r="M21" s="9"/>
+      <c r="M21" s="1"/>
       <c r="N21" s="9"/>
-      <c r="O21" s="55"/>
-      <c r="P21" s="54"/>
-      <c r="Q21" s="1"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="55"/>
+      <c r="Q21" s="54"/>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
-      <c r="U21" s="20"/>
-      <c r="V21" s="54"/>
-      <c r="W21" s="1"/>
-      <c r="X21" s="20"/>
-      <c r="Y21" s="7"/>
-      <c r="Z21" s="69"/>
+      <c r="U21" s="1"/>
+      <c r="V21" s="20"/>
+      <c r="W21" s="54"/>
+      <c r="X21" s="1"/>
+      <c r="Y21" s="20"/>
+      <c r="Z21" s="7"/>
       <c r="AA21" s="69"/>
       <c r="AB21" s="69"/>
       <c r="AC21" s="69"/>
-    </row>
-    <row r="22" spans="1:29">
+      <c r="AD21" s="69"/>
+    </row>
+    <row r="22" spans="1:30">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -9085,25 +9163,26 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="10"/>
+      <c r="M22" s="2"/>
       <c r="N22" s="10"/>
-      <c r="O22" s="57"/>
-      <c r="P22" s="56"/>
-      <c r="Q22" s="2"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="57"/>
+      <c r="Q22" s="56"/>
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
       <c r="T22" s="2"/>
-      <c r="U22" s="18"/>
-      <c r="V22" s="56"/>
-      <c r="W22" s="2"/>
-      <c r="X22" s="18"/>
-      <c r="Y22" s="8"/>
-      <c r="Z22" s="70"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="18"/>
+      <c r="W22" s="56"/>
+      <c r="X22" s="2"/>
+      <c r="Y22" s="18"/>
+      <c r="Z22" s="8"/>
       <c r="AA22" s="70"/>
       <c r="AB22" s="70"/>
       <c r="AC22" s="70"/>
-    </row>
-    <row r="23" spans="1:29">
+      <c r="AD22" s="70"/>
+    </row>
+    <row r="23" spans="1:30">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -9116,25 +9195,26 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
-      <c r="M23" s="9"/>
+      <c r="M23" s="1"/>
       <c r="N23" s="9"/>
-      <c r="O23" s="55"/>
-      <c r="P23" s="54"/>
-      <c r="Q23" s="1"/>
+      <c r="O23" s="9"/>
+      <c r="P23" s="55"/>
+      <c r="Q23" s="54"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
-      <c r="U23" s="20"/>
-      <c r="V23" s="54"/>
-      <c r="W23" s="1"/>
-      <c r="X23" s="20"/>
-      <c r="Y23" s="7"/>
-      <c r="Z23" s="69"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="20"/>
+      <c r="W23" s="54"/>
+      <c r="X23" s="1"/>
+      <c r="Y23" s="20"/>
+      <c r="Z23" s="7"/>
       <c r="AA23" s="69"/>
       <c r="AB23" s="69"/>
       <c r="AC23" s="69"/>
-    </row>
-    <row r="24" spans="1:29">
+      <c r="AD23" s="69"/>
+    </row>
+    <row r="24" spans="1:30">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -9147,25 +9227,26 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
-      <c r="M24" s="10"/>
+      <c r="M24" s="2"/>
       <c r="N24" s="10"/>
-      <c r="O24" s="57"/>
-      <c r="P24" s="56"/>
-      <c r="Q24" s="2"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="57"/>
+      <c r="Q24" s="56"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
-      <c r="U24" s="18"/>
-      <c r="V24" s="56"/>
-      <c r="W24" s="2"/>
-      <c r="X24" s="18"/>
-      <c r="Y24" s="8"/>
-      <c r="Z24" s="70"/>
+      <c r="U24" s="2"/>
+      <c r="V24" s="18"/>
+      <c r="W24" s="56"/>
+      <c r="X24" s="2"/>
+      <c r="Y24" s="18"/>
+      <c r="Z24" s="8"/>
       <c r="AA24" s="70"/>
       <c r="AB24" s="70"/>
       <c r="AC24" s="70"/>
-    </row>
-    <row r="25" spans="1:29">
+      <c r="AD24" s="70"/>
+    </row>
+    <row r="25" spans="1:30">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -9178,25 +9259,26 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
-      <c r="M25" s="9"/>
+      <c r="M25" s="1"/>
       <c r="N25" s="9"/>
-      <c r="O25" s="55"/>
-      <c r="P25" s="54"/>
-      <c r="Q25" s="1"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="55"/>
+      <c r="Q25" s="54"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
-      <c r="U25" s="20"/>
-      <c r="V25" s="54"/>
-      <c r="W25" s="1"/>
-      <c r="X25" s="20"/>
-      <c r="Y25" s="7"/>
-      <c r="Z25" s="69"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="20"/>
+      <c r="W25" s="54"/>
+      <c r="X25" s="1"/>
+      <c r="Y25" s="20"/>
+      <c r="Z25" s="7"/>
       <c r="AA25" s="69"/>
       <c r="AB25" s="69"/>
       <c r="AC25" s="69"/>
-    </row>
-    <row r="26" spans="1:29">
+      <c r="AD25" s="69"/>
+    </row>
+    <row r="26" spans="1:30">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -9209,25 +9291,26 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
-      <c r="M26" s="10"/>
+      <c r="M26" s="2"/>
       <c r="N26" s="10"/>
-      <c r="O26" s="57"/>
-      <c r="P26" s="56"/>
-      <c r="Q26" s="2"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="57"/>
+      <c r="Q26" s="56"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
       <c r="T26" s="2"/>
-      <c r="U26" s="18"/>
-      <c r="V26" s="56"/>
-      <c r="W26" s="2"/>
-      <c r="X26" s="18"/>
-      <c r="Y26" s="8"/>
-      <c r="Z26" s="70"/>
+      <c r="U26" s="2"/>
+      <c r="V26" s="18"/>
+      <c r="W26" s="56"/>
+      <c r="X26" s="2"/>
+      <c r="Y26" s="18"/>
+      <c r="Z26" s="8"/>
       <c r="AA26" s="70"/>
       <c r="AB26" s="70"/>
       <c r="AC26" s="70"/>
-    </row>
-    <row r="27" spans="1:29">
+      <c r="AD26" s="70"/>
+    </row>
+    <row r="27" spans="1:30">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -9240,25 +9323,26 @@
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
-      <c r="M27" s="9"/>
+      <c r="M27" s="1"/>
       <c r="N27" s="9"/>
-      <c r="O27" s="55"/>
-      <c r="P27" s="54"/>
-      <c r="Q27" s="1"/>
+      <c r="O27" s="9"/>
+      <c r="P27" s="55"/>
+      <c r="Q27" s="54"/>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
-      <c r="U27" s="20"/>
-      <c r="V27" s="54"/>
-      <c r="W27" s="1"/>
-      <c r="X27" s="20"/>
-      <c r="Y27" s="7"/>
-      <c r="Z27" s="69"/>
+      <c r="U27" s="1"/>
+      <c r="V27" s="20"/>
+      <c r="W27" s="54"/>
+      <c r="X27" s="1"/>
+      <c r="Y27" s="20"/>
+      <c r="Z27" s="7"/>
       <c r="AA27" s="69"/>
       <c r="AB27" s="69"/>
       <c r="AC27" s="69"/>
-    </row>
-    <row r="28" spans="1:29">
+      <c r="AD27" s="69"/>
+    </row>
+    <row r="28" spans="1:30">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -9271,25 +9355,26 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="M28" s="10"/>
+      <c r="M28" s="2"/>
       <c r="N28" s="10"/>
-      <c r="O28" s="57"/>
-      <c r="P28" s="56"/>
-      <c r="Q28" s="2"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="57"/>
+      <c r="Q28" s="56"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
-      <c r="U28" s="18"/>
-      <c r="V28" s="56"/>
-      <c r="W28" s="2"/>
-      <c r="X28" s="18"/>
-      <c r="Y28" s="8"/>
-      <c r="Z28" s="70"/>
+      <c r="U28" s="2"/>
+      <c r="V28" s="18"/>
+      <c r="W28" s="56"/>
+      <c r="X28" s="2"/>
+      <c r="Y28" s="18"/>
+      <c r="Z28" s="8"/>
       <c r="AA28" s="70"/>
       <c r="AB28" s="70"/>
       <c r="AC28" s="70"/>
-    </row>
-    <row r="29" spans="1:29">
+      <c r="AD28" s="70"/>
+    </row>
+    <row r="29" spans="1:30">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -9302,25 +9387,26 @@
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
-      <c r="M29" s="9"/>
+      <c r="M29" s="1"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="55"/>
-      <c r="P29" s="54"/>
-      <c r="Q29" s="1"/>
+      <c r="O29" s="9"/>
+      <c r="P29" s="55"/>
+      <c r="Q29" s="54"/>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
-      <c r="U29" s="20"/>
-      <c r="V29" s="54"/>
-      <c r="W29" s="1"/>
-      <c r="X29" s="20"/>
-      <c r="Y29" s="7"/>
-      <c r="Z29" s="69"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="20"/>
+      <c r="W29" s="54"/>
+      <c r="X29" s="1"/>
+      <c r="Y29" s="20"/>
+      <c r="Z29" s="7"/>
       <c r="AA29" s="69"/>
       <c r="AB29" s="69"/>
       <c r="AC29" s="69"/>
-    </row>
-    <row r="30" spans="1:29">
+      <c r="AD29" s="69"/>
+    </row>
+    <row r="30" spans="1:30">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -9333,25 +9419,26 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
-      <c r="M30" s="10"/>
+      <c r="M30" s="2"/>
       <c r="N30" s="10"/>
-      <c r="O30" s="57"/>
-      <c r="P30" s="56"/>
-      <c r="Q30" s="2"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="57"/>
+      <c r="Q30" s="56"/>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
       <c r="T30" s="2"/>
-      <c r="U30" s="18"/>
-      <c r="V30" s="56"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="18"/>
-      <c r="Y30" s="8"/>
-      <c r="Z30" s="70"/>
+      <c r="U30" s="2"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="56"/>
+      <c r="X30" s="2"/>
+      <c r="Y30" s="18"/>
+      <c r="Z30" s="8"/>
       <c r="AA30" s="70"/>
       <c r="AB30" s="70"/>
       <c r="AC30" s="70"/>
-    </row>
-    <row r="31" spans="1:29">
+      <c r="AD30" s="70"/>
+    </row>
+    <row r="31" spans="1:30">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -9364,25 +9451,26 @@
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
-      <c r="M31" s="9"/>
+      <c r="M31" s="1"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="55"/>
-      <c r="P31" s="54"/>
-      <c r="Q31" s="1"/>
+      <c r="O31" s="9"/>
+      <c r="P31" s="55"/>
+      <c r="Q31" s="54"/>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
-      <c r="U31" s="20"/>
-      <c r="V31" s="54"/>
-      <c r="W31" s="1"/>
-      <c r="X31" s="20"/>
-      <c r="Y31" s="7"/>
-      <c r="Z31" s="69"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="20"/>
+      <c r="W31" s="54"/>
+      <c r="X31" s="1"/>
+      <c r="Y31" s="20"/>
+      <c r="Z31" s="7"/>
       <c r="AA31" s="69"/>
       <c r="AB31" s="69"/>
       <c r="AC31" s="69"/>
-    </row>
-    <row r="32" spans="1:29">
+      <c r="AD31" s="69"/>
+    </row>
+    <row r="32" spans="1:30">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -9395,25 +9483,26 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
-      <c r="M32" s="10"/>
+      <c r="M32" s="2"/>
       <c r="N32" s="10"/>
-      <c r="O32" s="57"/>
-      <c r="P32" s="56"/>
-      <c r="Q32" s="2"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="57"/>
+      <c r="Q32" s="56"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
       <c r="T32" s="2"/>
-      <c r="U32" s="18"/>
-      <c r="V32" s="56"/>
-      <c r="W32" s="2"/>
-      <c r="X32" s="18"/>
-      <c r="Y32" s="8"/>
-      <c r="Z32" s="70"/>
+      <c r="U32" s="2"/>
+      <c r="V32" s="18"/>
+      <c r="W32" s="56"/>
+      <c r="X32" s="2"/>
+      <c r="Y32" s="18"/>
+      <c r="Z32" s="8"/>
       <c r="AA32" s="70"/>
       <c r="AB32" s="70"/>
       <c r="AC32" s="70"/>
-    </row>
-    <row r="33" spans="1:29">
+      <c r="AD32" s="70"/>
+    </row>
+    <row r="33" spans="1:30">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -9426,25 +9515,26 @@
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
-      <c r="M33" s="9"/>
+      <c r="M33" s="1"/>
       <c r="N33" s="9"/>
-      <c r="O33" s="55"/>
-      <c r="P33" s="54"/>
-      <c r="Q33" s="1"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="55"/>
+      <c r="Q33" s="54"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
       <c r="T33" s="1"/>
-      <c r="U33" s="20"/>
-      <c r="V33" s="54"/>
-      <c r="W33" s="1"/>
-      <c r="X33" s="20"/>
-      <c r="Y33" s="7"/>
-      <c r="Z33" s="69"/>
+      <c r="U33" s="1"/>
+      <c r="V33" s="20"/>
+      <c r="W33" s="54"/>
+      <c r="X33" s="1"/>
+      <c r="Y33" s="20"/>
+      <c r="Z33" s="7"/>
       <c r="AA33" s="69"/>
       <c r="AB33" s="69"/>
       <c r="AC33" s="69"/>
-    </row>
-    <row r="34" spans="1:29">
+      <c r="AD33" s="69"/>
+    </row>
+    <row r="34" spans="1:30">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -9457,25 +9547,26 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
-      <c r="M34" s="10"/>
+      <c r="M34" s="2"/>
       <c r="N34" s="10"/>
-      <c r="O34" s="57"/>
-      <c r="P34" s="56"/>
-      <c r="Q34" s="2"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="57"/>
+      <c r="Q34" s="56"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
       <c r="T34" s="2"/>
-      <c r="U34" s="18"/>
-      <c r="V34" s="56"/>
-      <c r="W34" s="2"/>
-      <c r="X34" s="18"/>
-      <c r="Y34" s="8"/>
-      <c r="Z34" s="70"/>
+      <c r="U34" s="2"/>
+      <c r="V34" s="18"/>
+      <c r="W34" s="56"/>
+      <c r="X34" s="2"/>
+      <c r="Y34" s="18"/>
+      <c r="Z34" s="8"/>
       <c r="AA34" s="70"/>
       <c r="AB34" s="70"/>
       <c r="AC34" s="70"/>
-    </row>
-    <row r="35" spans="1:29">
+      <c r="AD34" s="70"/>
+    </row>
+    <row r="35" spans="1:30">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -9488,25 +9579,26 @@
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
-      <c r="M35" s="9"/>
+      <c r="M35" s="1"/>
       <c r="N35" s="9"/>
-      <c r="O35" s="55"/>
-      <c r="P35" s="54"/>
-      <c r="Q35" s="1"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="55"/>
+      <c r="Q35" s="54"/>
       <c r="R35" s="1"/>
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
-      <c r="U35" s="20"/>
-      <c r="V35" s="54"/>
-      <c r="W35" s="1"/>
-      <c r="X35" s="20"/>
-      <c r="Y35" s="7"/>
-      <c r="Z35" s="69"/>
+      <c r="U35" s="1"/>
+      <c r="V35" s="20"/>
+      <c r="W35" s="54"/>
+      <c r="X35" s="1"/>
+      <c r="Y35" s="20"/>
+      <c r="Z35" s="7"/>
       <c r="AA35" s="69"/>
       <c r="AB35" s="69"/>
       <c r="AC35" s="69"/>
-    </row>
-    <row r="36" spans="1:29">
+      <c r="AD35" s="69"/>
+    </row>
+    <row r="36" spans="1:30">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -9519,25 +9611,26 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
-      <c r="M36" s="10"/>
+      <c r="M36" s="2"/>
       <c r="N36" s="10"/>
-      <c r="O36" s="57"/>
-      <c r="P36" s="56"/>
-      <c r="Q36" s="2"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="57"/>
+      <c r="Q36" s="56"/>
       <c r="R36" s="2"/>
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
-      <c r="U36" s="18"/>
-      <c r="V36" s="56"/>
-      <c r="W36" s="2"/>
-      <c r="X36" s="18"/>
-      <c r="Y36" s="8"/>
-      <c r="Z36" s="70"/>
+      <c r="U36" s="2"/>
+      <c r="V36" s="18"/>
+      <c r="W36" s="56"/>
+      <c r="X36" s="2"/>
+      <c r="Y36" s="18"/>
+      <c r="Z36" s="8"/>
       <c r="AA36" s="70"/>
       <c r="AB36" s="70"/>
       <c r="AC36" s="70"/>
-    </row>
-    <row r="37" spans="1:29">
+      <c r="AD36" s="70"/>
+    </row>
+    <row r="37" spans="1:30">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -9550,25 +9643,26 @@
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
-      <c r="M37" s="9"/>
+      <c r="M37" s="1"/>
       <c r="N37" s="9"/>
-      <c r="O37" s="55"/>
-      <c r="P37" s="54"/>
-      <c r="Q37" s="1"/>
+      <c r="O37" s="9"/>
+      <c r="P37" s="55"/>
+      <c r="Q37" s="54"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
-      <c r="U37" s="20"/>
-      <c r="V37" s="54"/>
-      <c r="W37" s="1"/>
-      <c r="X37" s="20"/>
-      <c r="Y37" s="7"/>
-      <c r="Z37" s="69"/>
+      <c r="U37" s="1"/>
+      <c r="V37" s="20"/>
+      <c r="W37" s="54"/>
+      <c r="X37" s="1"/>
+      <c r="Y37" s="20"/>
+      <c r="Z37" s="7"/>
       <c r="AA37" s="69"/>
       <c r="AB37" s="69"/>
       <c r="AC37" s="69"/>
-    </row>
-    <row r="38" spans="1:29">
+      <c r="AD37" s="69"/>
+    </row>
+    <row r="38" spans="1:30">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -9581,25 +9675,26 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
-      <c r="M38" s="10"/>
+      <c r="M38" s="2"/>
       <c r="N38" s="10"/>
-      <c r="O38" s="57"/>
-      <c r="P38" s="56"/>
-      <c r="Q38" s="2"/>
+      <c r="O38" s="10"/>
+      <c r="P38" s="57"/>
+      <c r="Q38" s="56"/>
       <c r="R38" s="2"/>
       <c r="S38" s="2"/>
       <c r="T38" s="2"/>
-      <c r="U38" s="18"/>
-      <c r="V38" s="56"/>
-      <c r="W38" s="2"/>
-      <c r="X38" s="18"/>
-      <c r="Y38" s="8"/>
-      <c r="Z38" s="70"/>
+      <c r="U38" s="2"/>
+      <c r="V38" s="18"/>
+      <c r="W38" s="56"/>
+      <c r="X38" s="2"/>
+      <c r="Y38" s="18"/>
+      <c r="Z38" s="8"/>
       <c r="AA38" s="70"/>
       <c r="AB38" s="70"/>
       <c r="AC38" s="70"/>
-    </row>
-    <row r="39" spans="1:29">
+      <c r="AD38" s="70"/>
+    </row>
+    <row r="39" spans="1:30">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -9612,25 +9707,26 @@
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
-      <c r="M39" s="9"/>
+      <c r="M39" s="1"/>
       <c r="N39" s="9"/>
-      <c r="O39" s="55"/>
-      <c r="P39" s="54"/>
-      <c r="Q39" s="1"/>
+      <c r="O39" s="9"/>
+      <c r="P39" s="55"/>
+      <c r="Q39" s="54"/>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
       <c r="T39" s="1"/>
-      <c r="U39" s="20"/>
-      <c r="V39" s="54"/>
-      <c r="W39" s="1"/>
-      <c r="X39" s="20"/>
-      <c r="Y39" s="7"/>
-      <c r="Z39" s="69"/>
+      <c r="U39" s="1"/>
+      <c r="V39" s="20"/>
+      <c r="W39" s="54"/>
+      <c r="X39" s="1"/>
+      <c r="Y39" s="20"/>
+      <c r="Z39" s="7"/>
       <c r="AA39" s="69"/>
       <c r="AB39" s="69"/>
       <c r="AC39" s="69"/>
-    </row>
-    <row r="40" spans="1:29">
+      <c r="AD39" s="69"/>
+    </row>
+    <row r="40" spans="1:30">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -9643,25 +9739,26 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
-      <c r="M40" s="10"/>
+      <c r="M40" s="2"/>
       <c r="N40" s="10"/>
-      <c r="O40" s="57"/>
-      <c r="P40" s="56"/>
-      <c r="Q40" s="2"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="57"/>
+      <c r="Q40" s="56"/>
       <c r="R40" s="2"/>
       <c r="S40" s="2"/>
       <c r="T40" s="2"/>
-      <c r="U40" s="18"/>
-      <c r="V40" s="56"/>
-      <c r="W40" s="2"/>
-      <c r="X40" s="18"/>
-      <c r="Y40" s="8"/>
-      <c r="Z40" s="70"/>
+      <c r="U40" s="2"/>
+      <c r="V40" s="18"/>
+      <c r="W40" s="56"/>
+      <c r="X40" s="2"/>
+      <c r="Y40" s="18"/>
+      <c r="Z40" s="8"/>
       <c r="AA40" s="70"/>
       <c r="AB40" s="70"/>
       <c r="AC40" s="70"/>
-    </row>
-    <row r="41" spans="1:29">
+      <c r="AD40" s="70"/>
+    </row>
+    <row r="41" spans="1:30">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -9674,25 +9771,26 @@
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
-      <c r="M41" s="9"/>
+      <c r="M41" s="1"/>
       <c r="N41" s="9"/>
-      <c r="O41" s="55"/>
-      <c r="P41" s="54"/>
-      <c r="Q41" s="1"/>
+      <c r="O41" s="9"/>
+      <c r="P41" s="55"/>
+      <c r="Q41" s="54"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
       <c r="T41" s="1"/>
-      <c r="U41" s="20"/>
-      <c r="V41" s="54"/>
-      <c r="W41" s="1"/>
-      <c r="X41" s="20"/>
-      <c r="Y41" s="7"/>
-      <c r="Z41" s="69"/>
+      <c r="U41" s="1"/>
+      <c r="V41" s="20"/>
+      <c r="W41" s="54"/>
+      <c r="X41" s="1"/>
+      <c r="Y41" s="20"/>
+      <c r="Z41" s="7"/>
       <c r="AA41" s="69"/>
       <c r="AB41" s="69"/>
       <c r="AC41" s="69"/>
-    </row>
-    <row r="42" spans="1:29">
+      <c r="AD41" s="69"/>
+    </row>
+    <row r="42" spans="1:30">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -9705,25 +9803,26 @@
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
-      <c r="M42" s="10"/>
+      <c r="M42" s="2"/>
       <c r="N42" s="10"/>
-      <c r="O42" s="57"/>
-      <c r="P42" s="56"/>
-      <c r="Q42" s="2"/>
+      <c r="O42" s="10"/>
+      <c r="P42" s="57"/>
+      <c r="Q42" s="56"/>
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
       <c r="T42" s="2"/>
-      <c r="U42" s="18"/>
-      <c r="V42" s="56"/>
-      <c r="W42" s="2"/>
-      <c r="X42" s="18"/>
-      <c r="Y42" s="8"/>
-      <c r="Z42" s="70"/>
+      <c r="U42" s="2"/>
+      <c r="V42" s="18"/>
+      <c r="W42" s="56"/>
+      <c r="X42" s="2"/>
+      <c r="Y42" s="18"/>
+      <c r="Z42" s="8"/>
       <c r="AA42" s="70"/>
       <c r="AB42" s="70"/>
       <c r="AC42" s="70"/>
-    </row>
-    <row r="43" spans="1:29">
+      <c r="AD42" s="70"/>
+    </row>
+    <row r="43" spans="1:30">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -9736,25 +9835,26 @@
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
-      <c r="M43" s="9"/>
+      <c r="M43" s="1"/>
       <c r="N43" s="9"/>
-      <c r="O43" s="55"/>
-      <c r="P43" s="54"/>
-      <c r="Q43" s="1"/>
+      <c r="O43" s="9"/>
+      <c r="P43" s="55"/>
+      <c r="Q43" s="54"/>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
       <c r="T43" s="1"/>
-      <c r="U43" s="20"/>
-      <c r="V43" s="54"/>
-      <c r="W43" s="1"/>
-      <c r="X43" s="20"/>
-      <c r="Y43" s="7"/>
-      <c r="Z43" s="69"/>
+      <c r="U43" s="1"/>
+      <c r="V43" s="20"/>
+      <c r="W43" s="54"/>
+      <c r="X43" s="1"/>
+      <c r="Y43" s="20"/>
+      <c r="Z43" s="7"/>
       <c r="AA43" s="69"/>
       <c r="AB43" s="69"/>
       <c r="AC43" s="69"/>
-    </row>
-    <row r="44" spans="1:29">
+      <c r="AD43" s="69"/>
+    </row>
+    <row r="44" spans="1:30">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -9767,25 +9867,26 @@
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
-      <c r="M44" s="10"/>
+      <c r="M44" s="2"/>
       <c r="N44" s="10"/>
-      <c r="O44" s="57"/>
-      <c r="P44" s="56"/>
-      <c r="Q44" s="2"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="57"/>
+      <c r="Q44" s="56"/>
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="U44" s="18"/>
-      <c r="V44" s="56"/>
-      <c r="W44" s="2"/>
-      <c r="X44" s="18"/>
-      <c r="Y44" s="8"/>
-      <c r="Z44" s="70"/>
+      <c r="U44" s="2"/>
+      <c r="V44" s="18"/>
+      <c r="W44" s="56"/>
+      <c r="X44" s="2"/>
+      <c r="Y44" s="18"/>
+      <c r="Z44" s="8"/>
       <c r="AA44" s="70"/>
       <c r="AB44" s="70"/>
       <c r="AC44" s="70"/>
-    </row>
-    <row r="45" spans="1:29">
+      <c r="AD44" s="70"/>
+    </row>
+    <row r="45" spans="1:30">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -9798,25 +9899,26 @@
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
-      <c r="M45" s="9"/>
+      <c r="M45" s="1"/>
       <c r="N45" s="9"/>
-      <c r="O45" s="55"/>
-      <c r="P45" s="54"/>
-      <c r="Q45" s="1"/>
+      <c r="O45" s="9"/>
+      <c r="P45" s="55"/>
+      <c r="Q45" s="54"/>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
       <c r="T45" s="1"/>
-      <c r="U45" s="20"/>
-      <c r="V45" s="54"/>
-      <c r="W45" s="1"/>
-      <c r="X45" s="20"/>
-      <c r="Y45" s="7"/>
-      <c r="Z45" s="69"/>
+      <c r="U45" s="1"/>
+      <c r="V45" s="20"/>
+      <c r="W45" s="54"/>
+      <c r="X45" s="1"/>
+      <c r="Y45" s="20"/>
+      <c r="Z45" s="7"/>
       <c r="AA45" s="69"/>
       <c r="AB45" s="69"/>
       <c r="AC45" s="69"/>
-    </row>
-    <row r="46" spans="1:29">
+      <c r="AD45" s="69"/>
+    </row>
+    <row r="46" spans="1:30">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -9829,25 +9931,26 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
-      <c r="M46" s="10"/>
+      <c r="M46" s="2"/>
       <c r="N46" s="10"/>
-      <c r="O46" s="57"/>
-      <c r="P46" s="56"/>
-      <c r="Q46" s="2"/>
+      <c r="O46" s="10"/>
+      <c r="P46" s="57"/>
+      <c r="Q46" s="56"/>
       <c r="R46" s="2"/>
       <c r="S46" s="2"/>
       <c r="T46" s="2"/>
-      <c r="U46" s="18"/>
-      <c r="V46" s="56"/>
-      <c r="W46" s="2"/>
-      <c r="X46" s="18"/>
-      <c r="Y46" s="8"/>
-      <c r="Z46" s="70"/>
+      <c r="U46" s="2"/>
+      <c r="V46" s="18"/>
+      <c r="W46" s="56"/>
+      <c r="X46" s="2"/>
+      <c r="Y46" s="18"/>
+      <c r="Z46" s="8"/>
       <c r="AA46" s="70"/>
       <c r="AB46" s="70"/>
       <c r="AC46" s="70"/>
-    </row>
-    <row r="47" spans="1:29">
+      <c r="AD46" s="70"/>
+    </row>
+    <row r="47" spans="1:30">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -9860,25 +9963,26 @@
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
-      <c r="M47" s="9"/>
+      <c r="M47" s="1"/>
       <c r="N47" s="9"/>
-      <c r="O47" s="55"/>
-      <c r="P47" s="54"/>
-      <c r="Q47" s="1"/>
+      <c r="O47" s="9"/>
+      <c r="P47" s="55"/>
+      <c r="Q47" s="54"/>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
       <c r="T47" s="1"/>
-      <c r="U47" s="20"/>
-      <c r="V47" s="54"/>
-      <c r="W47" s="1"/>
-      <c r="X47" s="20"/>
-      <c r="Y47" s="7"/>
-      <c r="Z47" s="69"/>
+      <c r="U47" s="1"/>
+      <c r="V47" s="20"/>
+      <c r="W47" s="54"/>
+      <c r="X47" s="1"/>
+      <c r="Y47" s="20"/>
+      <c r="Z47" s="7"/>
       <c r="AA47" s="69"/>
       <c r="AB47" s="69"/>
       <c r="AC47" s="69"/>
-    </row>
-    <row r="48" spans="1:29">
+      <c r="AD47" s="69"/>
+    </row>
+    <row r="48" spans="1:30">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -9891,25 +9995,26 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
-      <c r="M48" s="10"/>
+      <c r="M48" s="2"/>
       <c r="N48" s="10"/>
-      <c r="O48" s="57"/>
-      <c r="P48" s="56"/>
-      <c r="Q48" s="2"/>
+      <c r="O48" s="10"/>
+      <c r="P48" s="57"/>
+      <c r="Q48" s="56"/>
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
       <c r="T48" s="2"/>
-      <c r="U48" s="18"/>
-      <c r="V48" s="56"/>
-      <c r="W48" s="2"/>
-      <c r="X48" s="18"/>
-      <c r="Y48" s="8"/>
-      <c r="Z48" s="70"/>
+      <c r="U48" s="2"/>
+      <c r="V48" s="18"/>
+      <c r="W48" s="56"/>
+      <c r="X48" s="2"/>
+      <c r="Y48" s="18"/>
+      <c r="Z48" s="8"/>
       <c r="AA48" s="70"/>
       <c r="AB48" s="70"/>
       <c r="AC48" s="70"/>
-    </row>
-    <row r="49" spans="1:29">
+      <c r="AD48" s="70"/>
+    </row>
+    <row r="49" spans="1:30">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -9922,25 +10027,26 @@
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
-      <c r="M49" s="9"/>
+      <c r="M49" s="1"/>
       <c r="N49" s="9"/>
-      <c r="O49" s="55"/>
-      <c r="P49" s="54"/>
-      <c r="Q49" s="1"/>
+      <c r="O49" s="9"/>
+      <c r="P49" s="55"/>
+      <c r="Q49" s="54"/>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
       <c r="T49" s="1"/>
-      <c r="U49" s="20"/>
-      <c r="V49" s="54"/>
-      <c r="W49" s="1"/>
-      <c r="X49" s="20"/>
-      <c r="Y49" s="7"/>
-      <c r="Z49" s="69"/>
+      <c r="U49" s="1"/>
+      <c r="V49" s="20"/>
+      <c r="W49" s="54"/>
+      <c r="X49" s="1"/>
+      <c r="Y49" s="20"/>
+      <c r="Z49" s="7"/>
       <c r="AA49" s="69"/>
       <c r="AB49" s="69"/>
       <c r="AC49" s="69"/>
-    </row>
-    <row r="50" spans="1:29">
+      <c r="AD49" s="69"/>
+    </row>
+    <row r="50" spans="1:30">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -9953,23 +10059,24 @@
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
-      <c r="M50" s="10"/>
+      <c r="M50" s="2"/>
       <c r="N50" s="10"/>
-      <c r="O50" s="57"/>
-      <c r="P50" s="56"/>
-      <c r="Q50" s="2"/>
+      <c r="O50" s="10"/>
+      <c r="P50" s="57"/>
+      <c r="Q50" s="56"/>
       <c r="R50" s="2"/>
       <c r="S50" s="2"/>
       <c r="T50" s="2"/>
-      <c r="U50" s="18"/>
-      <c r="V50" s="56"/>
-      <c r="W50" s="2"/>
-      <c r="X50" s="18"/>
-      <c r="Y50" s="8"/>
-      <c r="Z50" s="70"/>
+      <c r="U50" s="2"/>
+      <c r="V50" s="18"/>
+      <c r="W50" s="56"/>
+      <c r="X50" s="2"/>
+      <c r="Y50" s="18"/>
+      <c r="Z50" s="8"/>
       <c r="AA50" s="70"/>
       <c r="AB50" s="70"/>
       <c r="AC50" s="70"/>
+      <c r="AD50" s="70"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -9980,128 +10087,128 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2763D7D-3C9B-B343-A9BB-0DE28C00E50A}">
   <dimension ref="A1:Q50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="35.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.5" customWidth="1"/>
-    <col min="14" max="14" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.33203125" customWidth="1"/>
-    <col min="16" max="16" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.453125" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.36328125" customWidth="1"/>
+    <col min="16" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="122">
+    <row r="1" spans="1:17" ht="118.5">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E1" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1" s="36" t="s">
         <v>96</v>
-      </c>
-      <c r="F1" s="36" t="s">
-        <v>97</v>
       </c>
       <c r="G1" s="36" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="40" t="s">
+      <c r="J1" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="45" t="s">
+      <c r="K1" s="43" t="s">
+        <v>92</v>
+      </c>
+      <c r="L1" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="M1" s="72" t="s">
+        <v>134</v>
+      </c>
+      <c r="N1" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="P1" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q1" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="43" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="43" t="s">
-        <v>94</v>
-      </c>
-      <c r="M1" s="72" t="s">
-        <v>135</v>
-      </c>
-      <c r="N1" s="43" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="45" t="s">
-        <v>43</v>
-      </c>
-      <c r="P1" s="43" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q1" s="43" t="s">
+    </row>
+    <row r="2" spans="1:17" ht="13">
+      <c r="A2" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H2" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="L2" s="50" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
-      <c r="A2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="H2" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="51" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="L2" s="50" t="s">
-        <v>48</v>
-      </c>
       <c r="M2" s="50" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N2" s="50" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O2" s="51" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="P2" s="50" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q2" s="50" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -11024,76 +11131,76 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{427C6688-DB1C-B542-B242-F45BBB834AB0}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <sheetData>
-    <row r="1" spans="1:11" ht="105">
+    <row r="1" spans="1:11" ht="101">
       <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="35" t="s">
+        <v>119</v>
+      </c>
+      <c r="E1" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="F1" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="G1" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="G1" s="35" t="s">
+      <c r="H1" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="H1" s="35" t="s">
+      <c r="I1" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="35" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="13">
+      <c r="A2" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="I1" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="J1" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="K1" s="35" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G2" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="I2" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="H2" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="I2" s="13" t="s">
+      <c r="J2" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="J2" s="13" t="s">
-        <v>128</v>
-      </c>
       <c r="K2" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>